<commit_message>
Add CUMCM 2026 Problem C paper (Q1/Q2), README, and final results
- 2026数学建模国赛论文.docx: full paper for Q1/Q2 (LP model, HiGHS solver, sensitivity analysis)
- make_paper.py: paper generation script (python-docx)
- README.md: project overview, model, results, usage
- Restore C题/result1.xlsx with baseline parameters
- Remove obsolete scratch files (1.py, format2026.txt)
</commit_message>
<xml_diff>
--- a/C题/result1.xlsx
+++ b/C题/result1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="计划购电量" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="充放电量" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计划购电量" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="充放电量" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>